<commit_message>
Enhance Excel audit report with formatting and risk summary
</commit_message>
<xml_diff>
--- a/output/audit_risk_report.xlsx
+++ b/output/audit_risk_report.xlsx
@@ -7,20 +7,24 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Audit Results" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Audit Summary" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
-  <definedNames/>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Audit Results'!$A$1:$I$11</definedName>
+  </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
     <numFmt numFmtId="165" formatCode="YYYY-MM-DD HH:MM:SS"/>
+    <numFmt numFmtId="166" formatCode="$#,##0.00"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -28,13 +32,31 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b val="1"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F4CCCC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF2CC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D9EAD3"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -49,9 +71,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -126,6 +153,140 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Risk Distribution</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <barChart>
+        <barDir val="col"/>
+        <grouping val="clustered"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Audit Summary'!$A$5:$A$7</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Audit Summary'!$B$5:$B$7</f>
+            </numRef>
+          </val>
+        </ser>
+        <gapWidth val="150"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </barChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Risk Level</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Number of Journal Entries</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>3</col>
+      <colOff>0</colOff>
+      <row>1</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="5400000" cy="2700000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="1" name="Chart 1"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -419,49 +580,60 @@
   </sheetPr>
   <dimension ref="A1:I11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="21" customWidth="1" min="2" max="2"/>
+    <col width="9" customWidth="1" min="3" max="3"/>
+    <col width="21" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="45" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Journal_ID</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Posting_Date</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Account</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Description</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Amount</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Prepared_By</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Risk_Score</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Risk_Reasons</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Risk_Level</t>
         </is>
@@ -473,7 +645,7 @@
           <t>JE008</t>
         </is>
       </c>
-      <c r="B2" s="1" t="n">
+      <c r="B2" s="2" t="n">
         <v>46277</v>
       </c>
       <c r="C2" t="n">
@@ -484,7 +656,7 @@
           <t>Professional Fees</t>
         </is>
       </c>
-      <c r="E2" t="n">
+      <c r="E2" s="3" t="n">
         <v>10000</v>
       </c>
       <c r="F2" t="inlineStr">
@@ -500,7 +672,7 @@
           <t xml:space="preserve">Weekend Posting; Round Dollar; High Value; </t>
         </is>
       </c>
-      <c r="I2" t="inlineStr">
+      <c r="I2" s="4" t="inlineStr">
         <is>
           <t>High</t>
         </is>
@@ -512,7 +684,7 @@
           <t>JE002</t>
         </is>
       </c>
-      <c r="B3" s="1" t="n">
+      <c r="B3" s="2" t="n">
         <v>46267</v>
       </c>
       <c r="C3" t="n">
@@ -523,7 +695,7 @@
           <t>Consulting Services</t>
         </is>
       </c>
-      <c r="E3" t="n">
+      <c r="E3" s="3" t="n">
         <v>5000</v>
       </c>
       <c r="F3" t="inlineStr">
@@ -539,7 +711,7 @@
           <t xml:space="preserve">Round Dollar; High Value; </t>
         </is>
       </c>
-      <c r="I3" t="inlineStr">
+      <c r="I3" s="4" t="inlineStr">
         <is>
           <t>High</t>
         </is>
@@ -551,7 +723,7 @@
           <t>JE010</t>
         </is>
       </c>
-      <c r="B4" s="1" t="n">
+      <c r="B4" s="2" t="n">
         <v>46280</v>
       </c>
       <c r="C4" t="n">
@@ -562,7 +734,7 @@
           <t>Consulting Services</t>
         </is>
       </c>
-      <c r="E4" t="n">
+      <c r="E4" s="3" t="n">
         <v>5000</v>
       </c>
       <c r="F4" t="inlineStr">
@@ -578,7 +750,7 @@
           <t xml:space="preserve">Round Dollar; High Value; </t>
         </is>
       </c>
-      <c r="I4" t="inlineStr">
+      <c r="I4" s="4" t="inlineStr">
         <is>
           <t>High</t>
         </is>
@@ -590,7 +762,7 @@
           <t>JE004</t>
         </is>
       </c>
-      <c r="B5" s="1" t="n">
+      <c r="B5" s="2" t="n">
         <v>46271</v>
       </c>
       <c r="C5" t="n">
@@ -601,7 +773,7 @@
           <t>Equipment Repair</t>
         </is>
       </c>
-      <c r="E5" t="n">
+      <c r="E5" s="3" t="n">
         <v>8750</v>
       </c>
       <c r="F5" t="inlineStr">
@@ -617,7 +789,7 @@
           <t xml:space="preserve">Weekend Posting; High Value; </t>
         </is>
       </c>
-      <c r="I5" t="inlineStr">
+      <c r="I5" s="4" t="inlineStr">
         <is>
           <t>High</t>
         </is>
@@ -629,7 +801,7 @@
           <t>JE006</t>
         </is>
       </c>
-      <c r="B6" s="1" t="n">
+      <c r="B6" s="2" t="n">
         <v>46273</v>
       </c>
       <c r="C6" t="n">
@@ -640,7 +812,7 @@
           <t>Customer Payment</t>
         </is>
       </c>
-      <c r="E6" t="n">
+      <c r="E6" s="3" t="n">
         <v>2500</v>
       </c>
       <c r="F6" t="inlineStr">
@@ -656,7 +828,7 @@
           <t xml:space="preserve">Potential Duplicate; </t>
         </is>
       </c>
-      <c r="I6" t="inlineStr">
+      <c r="I6" s="4" t="inlineStr">
         <is>
           <t>High</t>
         </is>
@@ -668,7 +840,7 @@
           <t>JE005</t>
         </is>
       </c>
-      <c r="B7" s="1" t="n">
+      <c r="B7" s="2" t="n">
         <v>46273</v>
       </c>
       <c r="C7" t="n">
@@ -679,7 +851,7 @@
           <t>Customer Payment</t>
         </is>
       </c>
-      <c r="E7" t="n">
+      <c r="E7" s="3" t="n">
         <v>2500</v>
       </c>
       <c r="F7" t="inlineStr">
@@ -695,7 +867,7 @@
           <t xml:space="preserve">Potential Duplicate; </t>
         </is>
       </c>
-      <c r="I7" t="inlineStr">
+      <c r="I7" s="4" t="inlineStr">
         <is>
           <t>High</t>
         </is>
@@ -707,7 +879,7 @@
           <t>JE003</t>
         </is>
       </c>
-      <c r="B8" s="1" t="n">
+      <c r="B8" s="2" t="n">
         <v>46270</v>
       </c>
       <c r="C8" t="n">
@@ -718,7 +890,7 @@
           <t>Office Supplies</t>
         </is>
       </c>
-      <c r="E8" t="n">
+      <c r="E8" s="3" t="n">
         <v>1000</v>
       </c>
       <c r="F8" t="inlineStr">
@@ -734,7 +906,7 @@
           <t xml:space="preserve">Weekend Posting; Round Dollar; </t>
         </is>
       </c>
-      <c r="I8" t="inlineStr">
+      <c r="I8" s="5" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
@@ -746,7 +918,7 @@
           <t>JE001</t>
         </is>
       </c>
-      <c r="B9" s="1" t="n">
+      <c r="B9" s="2" t="n">
         <v>46266</v>
       </c>
       <c r="C9" t="n">
@@ -757,7 +929,7 @@
           <t>Office Supplies</t>
         </is>
       </c>
-      <c r="E9" t="n">
+      <c r="E9" s="3" t="n">
         <v>245.75</v>
       </c>
       <c r="F9" t="inlineStr">
@@ -769,7 +941,7 @@
         <v>0</v>
       </c>
       <c r="H9" t="inlineStr"/>
-      <c r="I9" t="inlineStr">
+      <c r="I9" s="6" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
@@ -781,7 +953,7 @@
           <t>JE007</t>
         </is>
       </c>
-      <c r="B10" s="1" t="n">
+      <c r="B10" s="2" t="n">
         <v>46275</v>
       </c>
       <c r="C10" t="n">
@@ -792,7 +964,7 @@
           <t>Travel Expense</t>
         </is>
       </c>
-      <c r="E10" t="n">
+      <c r="E10" s="3" t="n">
         <v>487.36</v>
       </c>
       <c r="F10" t="inlineStr">
@@ -804,7 +976,7 @@
         <v>0</v>
       </c>
       <c r="H10" t="inlineStr"/>
-      <c r="I10" t="inlineStr">
+      <c r="I10" s="6" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
@@ -816,7 +988,7 @@
           <t>JE009</t>
         </is>
       </c>
-      <c r="B11" s="1" t="n">
+      <c r="B11" s="2" t="n">
         <v>46279</v>
       </c>
       <c r="C11" t="n">
@@ -827,7 +999,7 @@
           <t>Office Supplies</t>
         </is>
       </c>
-      <c r="E11" t="n">
+      <c r="E11" s="3" t="n">
         <v>83.47</v>
       </c>
       <c r="F11" t="inlineStr">
@@ -839,13 +1011,107 @@
         <v>0</v>
       </c>
       <c r="H11" t="inlineStr"/>
-      <c r="I11" t="inlineStr">
+      <c r="I11" s="6" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:I11"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="9" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Metric</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Total Journal Entries</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Flagged Entries</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Flagged Percentage</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>70.00%</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>High Risk</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Medium Risk</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Low Risk</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>3</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>